<commit_message>
657 sk bağlı kaynak dosyası güncellendi
</commit_message>
<xml_diff>
--- a/Uygulamalar ve Kaynakları/APP_Flashcard/657_Kaynak.xlsx
+++ b/Uygulamalar ve Kaynakları/APP_Flashcard/657_Kaynak.xlsx
@@ -18,6 +18,8 @@
     <definedName name="_ftn1" localSheetId="0">Sayfa1!$A$19</definedName>
     <definedName name="_ftnref1" localSheetId="0">Sayfa1!$A$16</definedName>
     <definedName name="_Toc235899280" localSheetId="0">Sayfa1!$A$44</definedName>
+    <definedName name="_Toc235899294" localSheetId="0">Sayfa1!$A$60</definedName>
+    <definedName name="_Toc235899296" localSheetId="0">Sayfa1!$A$61</definedName>
   </definedNames>
   <calcPr calcId="0"/>
   <extLst>
@@ -29,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="97">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="117">
   <si>
     <t>Bilgi edinme değerlendirme kurulu bir itirazı ne kadar sürede karara bağlar?</t>
   </si>
@@ -511,6 +513,66 @@
   </si>
   <si>
     <t xml:space="preserve">atamaya yetkili </t>
+  </si>
+  <si>
+    <t>Yer değiştirme suretiyle yapılan atanmalarda Olağanüstü Hal Bölgesine dahil illerle bu illere mücavir olarak belirlenen illerde görevli olanlara …..</t>
+  </si>
+  <si>
+    <t>% 60'ı,</t>
+  </si>
+  <si>
+    <t>Yer değiştirme suretiyle yapılan atanmalarda Kalkınmada 1 inci derecede öncelikli yörelerde görevli olanlara …..</t>
+  </si>
+  <si>
+    <t xml:space="preserve">% 50'si, </t>
+  </si>
+  <si>
+    <t>Yer değiştirme suretiyle yapılan atanmalarda Kalkınmada 2 nci derecede öncelikli yörelerde görevli olanlara …..</t>
+  </si>
+  <si>
+    <t xml:space="preserve">% 25'i, </t>
+  </si>
+  <si>
+    <t>Eşleri diğer yörelerde görevli olanlar ise ….. izinli sayılır.</t>
+  </si>
+  <si>
+    <t>ücretsiz</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yer değiştirme suretiyle yapılan atanmalarda kadroları eşlerinin görevlendirme süresiyle sınırlı olarak saklı tutulur. Ancak, bu süre memuriyet boyunca …. yılı hiç bir surette geçemez. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yer değiştirme suretiyle yapılan atanmalarda …. ilerlemesi; ….. ve diğer bütün hakları ve yükümlülükleri devam eder. </t>
+  </si>
+  <si>
+    <t>kademe - emeklilik</t>
+  </si>
+  <si>
+    <t>Yer değiştirme suretiyle yapılan atanmalarda ücretsiz izin verilenlerin bu sürelerinin emeklilikten sayılabilmesi için …….. karşılıklarının her ay kendileri tarafından T.C. Emekli Sandığına yatırılması gerekir.</t>
+  </si>
+  <si>
+    <t>kesenek ve kurum</t>
+  </si>
+  <si>
+    <t>Memurların atanamayacakları yerler ve bu yerlerdeki görevler ile kurumların özellik arz eden görevlerine atanabilmeleri için hangi kademelerde ne kadar hizmet etmeleri gerektiği ve yer değiştirme ile ilgili atama esasları ..... hazırlanacak bir yönetmelikle belirlenir</t>
+  </si>
+  <si>
+    <t>Memurların bir kurumdan diğerine nakillerinde Kazanılmış hak derecelerinin altındaki derecelere atanabilmeleri için ise atanacakları kadro derecesi ile kazanılmış hak dereceleri arasındaki farkın ….. dereceden çok olmaması ve memurların ... de şarttır</t>
+  </si>
+  <si>
+    <t>3 - isteği</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Memurların kurumlarınca görevlerinin ve yerlerinin değiştirilmesinde; Memurlar istekleri ile, kurumlarında kazanılmış hak derecelerinin en çok …. altında aynı veya başka yerlerdeki kadrolara atanabilirler. </t>
+  </si>
+  <si>
+    <t>üç derece</t>
+  </si>
+  <si>
+    <t>Yabancı bir memleket veya uluslararası kuruluşta hizmet almada; ) memuriyeti süresince yabancı memleketlerin resmî kurumlarında ya da Cumhurbaşkanınca belirlenen yurtdışındaki kuruluşlarda ....,  uluslararası kuruluşlarda ..... kadar aylıksız izin verilebilir.</t>
+  </si>
+  <si>
+    <t>on yıla -  yirmibir yıla</t>
   </si>
 </sst>
 </file>
@@ -752,7 +814,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B51"/>
+  <dimension ref="A1:B62"/>
   <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="15.6"/>
   <cols>
     <col min="1" max="1" width="85.6640625" style="3" customWidth="1"/>
@@ -1168,6 +1230,94 @@
         <v>96</v>
       </c>
     </row>
+    <row r="52" spans="1:2" ht="31.2">
+      <c r="A52" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="B52" s="3" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2" ht="31.2">
+      <c r="A53" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="B53" s="3" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2" ht="31.2">
+      <c r="A54" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="B54" s="3" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="55" spans="1:2">
+      <c r="A55" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="B55" s="3" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="56" spans="1:2" ht="31.2">
+      <c r="A56" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="B56" s="3">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="57" spans="1:2" ht="31.2">
+      <c r="A57" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="B57" s="3" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="58" spans="1:2" ht="46.8">
+      <c r="A58" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="B58" s="3" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="59" spans="1:2" ht="46.8">
+      <c r="A59" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="B59" s="3" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="60" spans="1:2" ht="46.8">
+      <c r="A60" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="B60" s="3" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="61" spans="1:2" ht="46.8">
+      <c r="A61" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="B61" s="3" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="62" spans="1:2" ht="46.8">
+      <c r="A62" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="B62" s="3" t="s">
+        <v>116</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.05277777777778" bottom="1.05277777777778" header="0.78749999999999998" footer="0.78749999999999998"/>
   <pageSetup paperSize="9" orientation="portrait" useFirstPageNumber="1" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>

</xml_diff>

<commit_message>
657 sk son hali eklendi
</commit_message>
<xml_diff>
--- a/Uygulamalar ve Kaynakları/APP_Flashcard/657_Kaynak.xlsx
+++ b/Uygulamalar ve Kaynakları/APP_Flashcard/657_Kaynak.xlsx
@@ -20,6 +20,7 @@
     <definedName name="_Toc235899280" localSheetId="0">Sayfa1!$A$44</definedName>
     <definedName name="_Toc235899294" localSheetId="0">Sayfa1!$A$60</definedName>
     <definedName name="_Toc235899296" localSheetId="0">Sayfa1!$A$61</definedName>
+    <definedName name="_Toc235899299" localSheetId="0">Sayfa1!$A$63</definedName>
   </definedNames>
   <calcPr calcId="0"/>
   <extLst>
@@ -31,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="117">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="381" uniqueCount="313">
   <si>
     <t>Bilgi edinme değerlendirme kurulu bir itirazı ne kadar sürede karara bağlar?</t>
   </si>
@@ -573,6 +574,669 @@
   </si>
   <si>
     <t>on yıla -  yirmibir yıla</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bilgilerini artırmak için yabancı memlekete gönderilenlerin hak ve yükümlülükleri kapsamında; Kadro karşılığı sözleşme ile istihdam edilenlerin sözleşmeleri devam eder ve (Şahsen özel burs sağlayan ve bu burstan istifade etmesi için kurumlarınca kendilerine maaşsız izin verilmesi uygun görülenler hariç) aylık ve diğer her türlü ödemeleri ile sözleşme ücretlerinin Kanuni kesintilerinden sonra kalan net tutarının ..... Kurumlarından alırlar. </t>
+  </si>
+  <si>
+    <t>% 60'ını</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bilgilerini artırmak için yabancı memlekete gönderilenlerin hak ve yükümlülükleri kapsamında; izin bitiminde yol süresi hariç ….. içinde görevlerine dönerler. </t>
+  </si>
+  <si>
+    <t>15 gün</t>
+  </si>
+  <si>
+    <t>Devlet memuru iken muvazzaf askerlik hizmetini yapmak üzere silah altına alınanlardan askerlik görevini tamamlayıp memuriyete dönmek isteyenler, terhis tarihinden itibaren .... içinde kurumlarına başvurmak ve kurumları da başvurma tarihinden itibaren azami ..... içinde ilgilileri göreve başlatmak zorundadırlar.</t>
+  </si>
+  <si>
+    <t>Bir görevin memurlar eliyle vekaleten yürütülmesi halinde ... vekalet asıldır.</t>
+  </si>
+  <si>
+    <t>aylıksız</t>
+  </si>
+  <si>
+    <t>Aynı kurumdan (…)ayrılmalar dolayısiyle atanan vekil memurlara vekalet görevinin 3 aydan fazla devam eden süresi için, kurum dışından veya açıktan atananlarla kurum içinden ilkokul öğretmenliğine atanan öğretmenler ile veznedarlık görevine atananlara göreve başladıkları tarihten itibaren .... ödenir.</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> vekalet aylığı</t>
+  </si>
+  <si>
+    <t>Açıktan vekil olarak atananlara, bir yılda yirmi günü geçmemek üzere çalıştıkları her ay için …. yıllık izin verilir. Bu iznin kullanımında, bir sonraki yıla devredilme hâli dışında Devlet memurları için öngörülen hükümler uygulanır.</t>
+  </si>
+  <si>
+    <t>iki gün</t>
+  </si>
+  <si>
+    <t>Bu Kanuna tabi kurumlarda, ikinci görev …. bu kurumlardan her ne ad ile olursa olsun para ….  ve yarar …..</t>
+  </si>
+  <si>
+    <t>verilemez - ödenemez - sağlanamaz.</t>
+  </si>
+  <si>
+    <t>Sermayesinin tamamı Devlet tarafından verilmek suretiyle kurulan iktisadi kurumlar ile sermayesinin yarısından fazlası Devlete ait bankalarda, ikinci görev …. bu kurumlardan her ne ad ile olursa olsun para ….  ve yarar …..</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Özel kanunlarla veya Cumhurbaşkanlığı kararnameleriyle kurulan banka ve kuruluşlarda, </t>
+    </r>
+    <r>
+      <rPr>
+        <vertAlign val="superscript"/>
+        <sz val="12"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+        <charset val="162"/>
+      </rPr>
+      <t>ikinci görev …. bu kurumlardan her ne ad ile olursa olsun para ….  ve yarar …..</t>
+    </r>
+  </si>
+  <si>
+    <t>Ücretle okutulacak ders saatlerinin sayısı, ders görevi alacakların nitelikleri ve diğer hususlar ….. kararı ile tespit olunur.</t>
+  </si>
+  <si>
+    <t>Cumhurbaşkanı</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Devlet memurlarına, vekalet görevi, ikinci görev veya ders görevlerinden ancak …. verilebilir. </t>
+  </si>
+  <si>
+    <t>birisi</t>
+  </si>
+  <si>
+    <t>Kadrosu kaldırılan memurlar, en geç …. içinde kendi kurumlarında niteliklerine uygun bir kadroya atanırlar.</t>
+  </si>
+  <si>
+    <t>altı ay</t>
+  </si>
+  <si>
+    <t>Memurların haftalık çalışma süresi genel olarak ... saattir.</t>
+  </si>
+  <si>
+    <r>
+      <t>…., yurt dışı kuruluşlarda hizmetin gerektirdiği hallerde, hafta tatilini Cumartesi ve Pazardan başka günler olarak tespit edebilir.</t>
+    </r>
+    <r>
+      <rPr>
+        <vertAlign val="superscript"/>
+        <sz val="12"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+        <charset val="162"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Günlük çalışmanın başlama ve bitme saatleri ile öğle dinlenme süresi, bölgelerin ve hizmetin özelliklerine göre merkezde …. illerde …. tarafından tesbit olunur.</t>
+    </r>
+    <r>
+      <rPr>
+        <vertAlign val="superscript"/>
+        <sz val="12"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+        <charset val="162"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+  </si>
+  <si>
+    <t>Cumhurbaşkanınca - valiler</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ancak, kadın memurlara; tabip raporunda belirtilmesi hâlinde hamileliğin yirmidördüncü haftasından önce ve her hâlde hamileliğin yirmidördüncü haftasından itibaren ve doğumdan sonraki …. süreyle gece nöbeti ve gece vardiyası görevi verilemez. </t>
+  </si>
+  <si>
+    <t>iki yıl</t>
+  </si>
+  <si>
+    <t>Engelli memurlara da isteği dışında gece nöbeti ve gece vardiyası görevi ……</t>
+  </si>
+  <si>
+    <t>verilemez</t>
+  </si>
+  <si>
+    <t>Devlet memurlarının yıllık izin süresi, hizmeti 1 yıldan on yıla kadar (On yıl dahil) olanlar için …., hizmeti on yıldan fazla olanlar için ... gündür. Zorunlu hallerde bu sürelere gidiş ve dönüş için en çok ….. gün eklenebilir.</t>
+  </si>
+  <si>
+    <t>yirmi gün - 30 - ikişer</t>
+  </si>
+  <si>
+    <t>Öğretmenler yaz tatili ile dinlenme tatillerinde izinli ….. Bunlara, hastalık ve diğer mazeret izinleri dışında, ayrıca yıllık izin …..</t>
+  </si>
+  <si>
+    <t>sayılırlar - verilmez.</t>
+  </si>
+  <si>
+    <t>Hizmetleri sırasında radyoaktif ışınlarla çalışan personele, her yıl yıllık izinlerine ilaveten ... aylık sağlık izni verilir.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kadın memura; doğumdan önce …, doğumdan sonra ... hafta olmak üzere toplam yirmidört hafta süreyle analık izni verilir. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">sekiz - onaltı </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Çoğul gebelik durumunda, doğum öncesi sekiz haftalık analık izni süresine ... hafta eklenir. </t>
+  </si>
+  <si>
+    <t>iki</t>
+  </si>
+  <si>
+    <t>on</t>
+  </si>
+  <si>
+    <t>Memura, eşinin doğum yapması hâlinde, isteği üzerine .. gün babalık izni; kendisinin veya çocuğunun evlenmesi ya da eşinin, çocuğunun, kendisinin veya eşinin ana, baba ve kardeşinin ölümü hâllerinde isteği üzerine ... gün izin verilir.</t>
+  </si>
+  <si>
+    <t>on - yedi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(A) ve (B) fıkralarında belirtilen hâller dışında, merkezde atamaya yetkili amir, ilde vali, ilçede kaymakam ve yurt dışında diplomatik misyon şefi tarafından, birim amirinin muvafakati ile bir yıl içinde toptan veya bölümler hâlinde, mazeretleri sebebiyle memurlara .... gün izin verilebilir. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kadın memura, çocuğunu emzirmesi için doğum sonrası analık izni süresinin bitim tarihinden itibaren ilk altı ayda günde .. saat, ikinci altı ayda günde …. saat süt izni verilir. </t>
+  </si>
+  <si>
+    <t>üç - birbuçuk</t>
+  </si>
+  <si>
+    <r>
+      <t>Memurlara; en az yüzde 70 oranında engelli ya da süreğen hastalığı olan çocuğunun (çocuğun evli olması durumunda eşinin de en az yüzde 70 oranında engelli olması kaydıyla) hastalanması hâlinde hastalık raporuna dayalı olarak ana veya babadan sadece biri tarafından kullanılması kaydıyla bir yıl içinde toptan veya bölümler hâlinde ... güne kadar mazeret izni verilir.</t>
+    </r>
+    <r>
+      <rPr>
+        <vertAlign val="superscript"/>
+        <sz val="12"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+        <charset val="162"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+  </si>
+  <si>
+    <t>onsekiz</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Memura, aylık ve özlük hakları korunarak, verilecek raporda gösterilecek lüzum üzerine, kanser, verem ve akıl hastalığı gibi uzun süreli bir tedaviye ihtiyaç gösteren hastalığı hâlinde .... aya kadar, diğer hastalık hâllerinde ise ... aya kadar izin verilir. </t>
+  </si>
+  <si>
+    <t>onsekiz - oniki</t>
+  </si>
+  <si>
+    <r>
+      <t>Memura</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+        <charset val="162"/>
+      </rPr>
+      <t>, 105 inci maddenin son fıkrası uyarınca verilen iznin bitiminden itibaren, sağlık kurulu raporuyla belgelendirilmesi şartıyla, istekleri üzerine …. aya kadar aylıksız izin verilebilir.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Doğum yapan memura</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+        <charset val="162"/>
+      </rPr>
+      <t>, 104 üncü madde uyarınca verilen doğum sonrası analık izni süresinin veya aynı maddenin (F) fıkrası uyarınca verilen izin süresinin bitiminden; eşi doğum yapan memura ise, doğum tarihinden itibaren istekleri üzerine .... aya kadar aylıksız izin verilir</t>
+    </r>
+  </si>
+  <si>
+    <t>yirmidört</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Memura, yıllık izinde esas alınan süreler itibarıyla beş hizmet yılını tamamlamış olması ve isteği hâlinde memuriyeti boyunca ve en fazla iki defada kullanılmak üzere, toplam …. kadar aylıksız izin verilebilir. </t>
+  </si>
+  <si>
+    <t>bir yıla</t>
+  </si>
+  <si>
+    <t>Özlük dosyalarının tutulma esasları ile özlük dosyalarında yer alacak belgelere ilişkin usûl ve esaslar... belirlenir.</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Devlet Personel Başkanlığınca</t>
+  </si>
+  <si>
+    <t>….; kurumların kuruluş ve görev özellikleri dikkate alınarak Devlet Personel Başkanlığı'nın görüşüne dayanılarak özel yönetmeliklerinde tayin ve tesbit edilecek amirlerdir.</t>
+  </si>
+  <si>
+    <t>Disiplin amirleri</t>
+  </si>
+  <si>
+    <t>Memura, görevinde ve davranışlarında daha dikkatli olması gerektiğinin yazı ile bildirilmesidir.</t>
+  </si>
+  <si>
+    <t>Uyarma</t>
+  </si>
+  <si>
+    <t>Verilen emir ve görevlerin tam ve zamanında yapılmasında, görev mahallinde kurumlarca belirlenen usul ve esasların yerine getirilmesinde, görevle ilgili resmi belge, araç ve gereçlerin korunması, kullanılması ve bakımında kayıtsızlık göstermek veya düzensiz davranmak,</t>
+  </si>
+  <si>
+    <t>Özürsüz veya izinsiz olarak göreve geç gelmek, erken ayrılmak, görev mahallini terketmek,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kurumca belirlenen tasarruf tedbirlerine riayet etmemek, </t>
+  </si>
+  <si>
+    <t>Usulsüz müracaat veya şikayette bulunmak,</t>
+  </si>
+  <si>
+    <t>Devlet memuru vakarına yakışmayan tutum ve davranışta bulunmak,</t>
+  </si>
+  <si>
+    <t>Görevine veya iş sahiplerine karşı kayıtsızlık göstermek veya ilgisiz kalmak,</t>
+  </si>
+  <si>
+    <t>Belirlenen kılık ve kıyafet hükümlerine aykırı davranmak,</t>
+  </si>
+  <si>
+    <t>Görevin işbirliği içinde yapılması ilkesine aykırı davranışlarda bulunmak.</t>
+  </si>
+  <si>
+    <t>Memura, görevinde ve davranışlarında kusurlu olduğunun yazı ile bildirilmesidir.(tanım)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kınama </t>
+  </si>
+  <si>
+    <t>Verilen emir ve görevlerin tam ve zamanında yapılmasında, görev mahallinde kurumlarca belirlenen usul ve esasların yerine getirilmesinde, görevle ilgili resmi belge, araç ve gereçlerin korunması, kullanılması ve bakımında kusurlu davranmak,</t>
+  </si>
+  <si>
+    <t>Eşlerinin, reşit olmayan veya mahcur olan çocuklarının kazanç getiren sürekli faaliyetlerini belirlenen sürede kurumuna bildirmemek,</t>
+  </si>
+  <si>
+    <t>Görev sırasında amire hal ve hareketi ile saygısız davranmak,</t>
+  </si>
+  <si>
+    <t>Hizmet dışında Devlet memurunun itibar ve güven duygusunu sarsacak nitelikte davranışlarda bulunmak,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Devlete ait resmi araç, gereç ve benzeri eşyayı özel işlerinde kullanmak, </t>
+  </si>
+  <si>
+    <t>Devlete ait resmî belge, araç, gereç ve benzeri eşyayı kaybetmek,</t>
+  </si>
+  <si>
+    <t>İş arkadaşlarına, maiyetindeki personele ve iş sahiplerine kötü muamelede bulunmak,</t>
+  </si>
+  <si>
+    <t>İş arkadaşlarına ve iş sahiplerine söz veya hareketle sataşmak,</t>
+  </si>
+  <si>
+    <t>Görev mahallinde genel ahlak ve edep dışı davranışlarda bulunmak ve bu tür yazı yazmak, işaret, resim ve benzeri şekiller çizmek ve yapmak,</t>
+  </si>
+  <si>
+    <t>Verilen emirlere itiraz etmek,</t>
+  </si>
+  <si>
+    <t>Borçlarını kasten ödemeyerek hakkında yasal yollara başvurulmasına neden olmak,</t>
+  </si>
+  <si>
+    <t>Kurumların huzur, sükûn ve çalışma düzenini bozmak.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yetkili olmadığı halde basına, haber ajanslarına veya radyo ve televizyon kurumlarına bilgi veya demeç vermek. </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Memurun, brüt aylığından 1/30 - 1/8 arasında kesinti yapılmasıdır. (tanım)</t>
+  </si>
+  <si>
+    <t>Aylıktan Kesme</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kasıtlı olarak; verilen emir ve görevleri tam ve zamanında yapmamak, görev mahallinde kurumlarca belirlenen usul ve esasları yerine getirmemek, görevle ilgili resmi belge, araç ve gereçleri korumamak, bakımını yapmamak, hor kullanmak, </t>
+  </si>
+  <si>
+    <t>Özürsüz olarak bir veya iki gün göreve gelmemek,</t>
+  </si>
+  <si>
+    <t>Devlete ait resmi belge, araç, gereç ve benzerlerini özel menfaat sağlamak için kullanmak,</t>
+  </si>
+  <si>
+    <t>Görevle ilgili konularda yükümlü olduğu kişilere yalan ve yanlış beyanda bulunmak,</t>
+  </si>
+  <si>
+    <t>Görev sırasında amirine sözle saygısızlık etmek,</t>
+  </si>
+  <si>
+    <t>Görev yeri sınırları içerisinde her hangi bir yerin toplantı, tören ve benzeri amaçlarla izinsiz olarak kullanılmasına yardımcı olmak,</t>
+  </si>
+  <si>
+    <t>Hizmet içinde Devlet memurunun itibar ve güven duygusunu sarsacak nitelikte davranışlarda bulunmak,</t>
+  </si>
+  <si>
+    <t>Fiilin ağırlık derecesine göre memurun, bulunduğu …. 1 - 3 yıl durdurulmasıdır.</t>
+  </si>
+  <si>
+    <t>kademede ilerlemesinin</t>
+  </si>
+  <si>
+    <t>Göreve sarhoş gelmek, görev yerinde alkollü içki içmek,</t>
+  </si>
+  <si>
+    <t>Kademe İlerlemesinin Durdurulması</t>
+  </si>
+  <si>
+    <t>Özürsüz ve kesintisiz 3 - 9 gün göreve gelmemek,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Görevi ile ilgili olarak her ne şekilde olursa olsun çıkar sağlamak, </t>
+  </si>
+  <si>
+    <t>Amirine veya maiyetindekilere karşı küçük düşürücü veya aşağılayıcı fiil ve hareketler yapmak,</t>
+  </si>
+  <si>
+    <t>Görev yeri sınırları içinde herhangi bir yeri toplantı, tören ve benzeri amaçlarla izinsiz kullanmak veya kullandırmak,</t>
+  </si>
+  <si>
+    <t>Gerçeğe aykırı rapor ve belge düzenlemek,</t>
+  </si>
+  <si>
+    <t>Ticaret yapmak veya Devlet memurlarına yasaklanan diğer kazanç getirici faaliyetlerde bulunmak,</t>
+  </si>
+  <si>
+    <t>Görevin yerine getirilmesinde dil, ırk, cinsiyet, siyasi düşünce, felsefi inanç, din ve mezhep ayrımı yapmak, kişilerin yarar veya zararını hedef tutan davranışlarda bulunmak,</t>
+  </si>
+  <si>
+    <t>Belirlenen durum ve sürelerde mal bildiriminde bulunmamak,</t>
+  </si>
+  <si>
+    <t>Açıklanması yasaklanan bilgileri açıklamak,</t>
+  </si>
+  <si>
+    <t>Amirine, maiyetindekilere, iş arkadaşları veya iş sahiplerine hakarette bulunmak veya bunları tehdit etmek,</t>
+  </si>
+  <si>
+    <t>Diplomatik statüsünden yararlanmak suretiyle yurt dışında, haklı bir sebep göstermeksizin ödeme kabiliyetinin üstünde borçlanmak ve borçlarını ödemedeki tutum ve davranışlarıyla Devlet itibarını zedelemek veya zorunlu bir sebebe dayanmaksızın borcunu ödemeden yurda dönmek,</t>
+  </si>
+  <si>
+    <t>Verilen görev ve emirleri kasten yapmamak,</t>
+  </si>
+  <si>
+    <t>Herhangi bir siyasi parti yararına veya zararına fiilen faaliyette bulunmak.</t>
+  </si>
+  <si>
+    <t>İdeolojik veya siyasi amaçlarla kurumların huzur, sükün ve çalışma düzenini bozmak, boykot, işgal, kamu hizmetlerinin yürütülmesini engelleme, işi yavaşlatma ve grev gibi eylemlere katılmak veya bu amaçlarla toplu olarak göreve gelmemek, bunları tahrik ve teşvik etmek veya yardımda bulunmak</t>
+  </si>
+  <si>
+    <t>Devlet Memurluğunda Çıkarma</t>
+  </si>
+  <si>
+    <t>Yasaklanmış her türlü yayını veya siyasi veya ideolojik amaçlı bildiri, afiş, pankart, bant ve benzerlerini basmak, çoğaltmak, dağıtmak veya bunları kurumların herhangi bir yerine asmak veya teşhir etmek,</t>
+  </si>
+  <si>
+    <t>Siyasi partiye girmek,</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Özürsüz olarak (...) bir yılda toplam 20 gün göreve gelmemek,</t>
+  </si>
+  <si>
+    <t>Savaş, olağanüstü hal veya genel afetlere ilişkin konularda amirlerin verdiği görev veya emirleri yapmamak,</t>
+  </si>
+  <si>
+    <t>Amirlerine, maiyetindekilere ve iş sahiplerine fiili tecavüzde bulunmak,</t>
+  </si>
+  <si>
+    <t>Memurluk sıfatı ile bağdaşmayacak nitelik ve derecede yüz kızartıcı ve utanç verici hareketlerde bulunmak,</t>
+  </si>
+  <si>
+    <t>Yetki almadan gizli bilgileri açıklamak,</t>
+  </si>
+  <si>
+    <t>Siyasi ve ideolojik eylemlerden arananları görev mahallinde gizlemek,</t>
+  </si>
+  <si>
+    <t>Yurt dışında Devletin itibarını düşürecek veya görev haysiyetini zedeleyecek tutum ve davranışlarda bulunmak,</t>
+  </si>
+  <si>
+    <t>5816 sayılı Atatürk Aleyhine İşlenen Suçlar Hakkındaki Kanuna aykırı fiilleri işlemek.</t>
+  </si>
+  <si>
+    <t>Terör örgütleriyle eylem birliği içerisinde olmak, bu örgütlere yardım etmek, kamu imkân ve kaynaklarını bu örgütleri desteklemeye yönelik kullanmak ya da kullandırmak, bu örgütlerin propagandasını yapmak.</t>
+  </si>
+  <si>
+    <t>Öğrenim durumları nedeniyle yükselebilecekleri kadroların son kademelerinde bulunan Devlet memurlarının, kademe ilerlemesinin durdurulması cezasının verilmesini gerektiren hallerde, brüt aylıklarının ….. kesilir ve tekerrüründe görevlerine son verilir.</t>
+  </si>
+  <si>
+    <t>¼’ü – ½’si</t>
+  </si>
+  <si>
+    <t>Uyarma, kınama ve aylıktan kesme cezaları ...... tarafından; kademe ilerlemesinin durdurulması cezası, memurun bağlı olduğu kurumdaki disiplin kurulunun kararı alındıktan sonra, atamaya yetkili amirler il disiplin kurullarının kararlarına dayanan hallerde valiler tarafından verilir</t>
+  </si>
+  <si>
+    <t xml:space="preserve">disiplin amirleri  </t>
+  </si>
+  <si>
+    <t>Devlet memurluğundan çıkarma cezası amirlerin bu yoldaki isteği üzerine, memurun bağlı bulunduğu kurumun…. kararı ile verilir.</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> yüksek disiplin kurulu</t>
+  </si>
+  <si>
+    <t>Disiplin kurulu ve yüksek disiplin kurulunun ayrı bir ceza tayinine yetkisi yoktur, cezayı …. veya ….</t>
+  </si>
+  <si>
+    <t>kabul - reddeder</t>
+  </si>
+  <si>
+    <t>(Disiplin cezası vermeye yetkili amir ve kurullar:)Ret halinde atamaya yetkili amirler ... gün içinde başka bir disiplin cezası vermekte serbesttirler.</t>
+  </si>
+  <si>
+    <t>Uyarma, kınama, aylıktan kesme ve kademe ilerlemesinin durdurulması cezalarında ... içinde disiplin soruşturmasına başlanmadığı takdirde zaman aşımına uğrar</t>
+  </si>
+  <si>
+    <t>bir ay</t>
+  </si>
+  <si>
+    <t>Memurluktan çıkarma cezasında …. içinde disiplin kovuşturmasına başlanmadığı takdirde zaman aşımına uğrar.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Disiplin cezasını gerektiren fiil ve hallerin işlendiği tarihten itibaren nihayet …. disiplin cezası verilmediği takdirde ceza verme yetkisi zamanaşımına uğrar. </t>
+  </si>
+  <si>
+    <t>iki yıl içinde</t>
+  </si>
+  <si>
+    <t>Disiplin amirleri uyarma, kınama ve aylıktan kesme cezalarını soruşturmanın tamamlandığı günden itibaren …. içinde vermek zorundadırlar.</t>
+  </si>
+  <si>
+    <t>Kademe ilerlemesinin durdurulması cezasını gerektiren hallerde soruşturma dosyası, kararını bildirmek üzere yetkili disiplin kuruluna ..... içinde tevdi edilir. Disiplin kurulu, dosyayı aldığı tarihten itibaren ..... içinde soruşturma evrakına göre kararını bildirir.</t>
+  </si>
+  <si>
+    <t>15 gün - 30 gün</t>
+  </si>
+  <si>
+    <t>Memurluktan çıkarma cezası için disiplin amirleri tarafından yaptırılan soruşturmaya ait dosya, memurun bağlı bulunduğu kurumun yüksek disiplin kuruluna tevdiinden itibaren azami …. içinde bu kurulca, karara bağlanır.</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> altı ay</t>
+  </si>
+  <si>
+    <t>Soruşturmayı yapanın veya yetkili disiplin kurulunun ….. az olmamak üzere verdiği süre içinde veya belirtilen bir tarihte savunmasını yapmıyan memur, savunma hakkından vazgeçmiş sayılır.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7 günden </t>
+  </si>
+  <si>
+    <t>Memurun ceza kanununa göre mahkûm olması veya olmaması halleri, ayrıca disiplin cezasının uygulanmasına engel ….</t>
+  </si>
+  <si>
+    <t>olamaz.</t>
+  </si>
+  <si>
+    <t>Verilen disiplin cezaları …., Devlet memurluğundan çıkarma cezası ayrıca ….. bildirilir</t>
+  </si>
+  <si>
+    <t>üst disiplin amirine - Devlet Personel Başkanlığına</t>
+  </si>
+  <si>
+    <t>Aylıktan kesme cezası ile tecziye edilenler ...., kademe ilerlemesinin durdurulması cezası ile tecziye edilenler ..... boyunca daire başkanı kadrolarına, daire başkanı kadrosunun dengi ve daha üstü kadrolara, bölge ve il teşkilatlarının en üst yönetici kadrolarına, düzenleyici ve denetleyici kurumların başkanlık ve üyeliklerine, vali ve büyükelçi kadrolarına atanamazlar.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5 yıl - 10 yıl </t>
+  </si>
+  <si>
+    <t>Disiplin kurulları  kuruluş, üyelerinin görev süresi, görüşme ve karar usulü, hangi memurlar hakkında karar verebilecekleri ve disiplin amirlerinin tayin ve tespitinde uygulanacak esaslar ile bunların yetki ve sorumlulukları gibi hususlar ..... çıkarılacak yönetmelikle düzenlenir</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Disiplin amirleri tarafından verilen uyarma, kınama ve aylıktan kesme cezalarına karşı ….., kademe ilerlemesinin durdurulması cezasına karşı …... itiraz edilebilir. </t>
+  </si>
+  <si>
+    <t>disiplin kuruluna - yüksek disiplin kuruluna</t>
+  </si>
+  <si>
+    <t>İtirazda süre, kararın ilgiliye tebliği tarihinden itibaren ... gündür. Süresi içinde itiraz edilmeyen disiplin cezaları kesinleşir.</t>
+  </si>
+  <si>
+    <t>yedi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">İtiraz mercileri, itiraz dilekçesi ile karar ve eklerinin kendilerine intikalinden itibaren ….içinde kararlarını vermek zorundadır. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">otuz gün </t>
+  </si>
+  <si>
+    <t>Görevden uzaklaştırmaya yetkililer şunlardır.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">a) Atamaya yetkili amirler;
+b) Bakanlık ve genel müdürlük müfettişleri;
+c) İllerde valiler;
+ç) İlçelerde kaymakamlar </t>
+  </si>
+  <si>
+    <t>Görevinden uzaklaştırılan Devlet memurları hakkında görevden uzaklaştırmayı izleyen ... iş günü içinde soruşturmaya başlanması şarttır.</t>
+  </si>
+  <si>
+    <t>Görevden uzaklaştırılan ve görevi ile ilgili olsun veya olmasın herhangi bir suçtan tutuklanan veya gözaltına alınan memurlara bu süre içinde aylıklarının ….. ödenir</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> üçte ikisi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Görevden uzaklaştırma; bir disiplin kovuşturması icabından olduğu takdirde en çok …. devam edebilir. </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 3 ay</t>
+  </si>
+  <si>
+    <t>Bu Kanuna tabi kurumlarda görevlendirilen memurlara hizmetlerinin karşılığında, kadroya dayanılarak ay itibariyle ödenen parayı,</t>
+  </si>
+  <si>
+    <t>Aylık</t>
+  </si>
+  <si>
+    <t>Niteliği ve çalışma şartları bakımından güç olan işlerde çalışanlara ödenen parayı,</t>
+  </si>
+  <si>
+    <t>İş güçlüğü zammı</t>
+  </si>
+  <si>
+    <t>Hayat ve sağlık için tahlike arz eden hizmetlerde çalışanlara ödenen parayı,</t>
+  </si>
+  <si>
+    <t>İş riski zammı</t>
+  </si>
+  <si>
+    <t>Bir göreve vekaleten atanan memurlara vekalet edilen görevin kadro derecesinin birinci kademesinin ...., açıktan atananlara ise (Köy ve kasaba imamlığı kadrolarına atananlara 146 ncı maddede yazılı asgari ücret aylık tutarından aşağı olmamak üzere) .... verilir</t>
+  </si>
+  <si>
+    <t>üçte biri - üçte ikisi</t>
+  </si>
+  <si>
+    <t>Kurumlar gerektiği takdirde personelini günlük çalışma saatleri dışında fazla çalışma ücreti vermeksizin ….. Bu durumda personele yaptırılacak fazla çalışmanın her ... saati için bir gün hesabı ile izin verilir.</t>
+  </si>
+  <si>
+    <t>çalıştırabilirler - sekiz</t>
+  </si>
+  <si>
+    <t>Fazla çalışmanın uygulama esas ve usulleri ….. ile ….. Bakanlığınca müştereken belirlenir.</t>
+  </si>
+  <si>
+    <t>Devlet Personel Başkanlığı - Maliye</t>
+  </si>
+  <si>
+    <t>Sürekli görevle yurt dışına gönderilen Devlet memurları, geçici görevle en çok …. süre ile merkeze çağrılabilir. Bu süre içinde aylığı katsayılı ödenir.</t>
+  </si>
+  <si>
+    <t>Yedek subay, yedek askeri memur ve yedek astsubay olanların rütbelerine ait aylıkları …... ödenir.</t>
+  </si>
+  <si>
+    <t>Milli Savunma Bakanlığınca</t>
+  </si>
+  <si>
+    <t>Devlet Memurlarından T. C. Emekli Sandığına tabi hizmeti 10 yıl ve daha fazla olanlara, istekleri üzerine Toplu Konut Fonundan özel şartlarla ve öncelikle konut kredisi …..</t>
+  </si>
+  <si>
+    <t>verilebilir.</t>
+  </si>
+  <si>
+    <t>verilir.</t>
+  </si>
+  <si>
+    <t>Evli bulunan Devlet memurlarına aile yardımı ödeneği …. (Aile yardımı ödeneği)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Geçici süreli görevlendirme süresi bir yılda …. ayı geçemez. </t>
+  </si>
+  <si>
+    <t>altı</t>
+  </si>
+  <si>
+    <t>Yurtdışında görevlendirilen güvenlik görevlileri için geçici görevlendirme süresi en çok ... yıldır; gerekli görülmesi hâlinde bu süre bir katına kadar uzatılabilir.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bu kanuna ekli IV sayılı cetvelde unvanları yazılı görevlerde bulunanlara hizalarında gösterilen gösterge rakamlarının memur aylıklarına uygulanan katsayı ile çarpımı sonucu bulunan miktarda .... ödenir. Makam tazminatı damga vergisi hariç herhangi bir vergiye tabi ... ve ödemelerde aylıklara ilişkin hükümler uygulanır. </t>
+  </si>
+  <si>
+    <t>makam tazminatı - tutulmaz</t>
+  </si>
+  <si>
+    <t>Makam tazminatı ödenmeleri her ay  …. Ödenir. İlgili kurum bu ödemeleri … aylık dönemler halinde faturası karşılığında … tahsil eder.</t>
+  </si>
+  <si>
+    <t>T.C. Emekli Sandığınca - 3 - Hazine</t>
+  </si>
+  <si>
+    <t xml:space="preserve">68 yaşını geçmemek kaydıyla Müsteşar …. olarak çalıştırılabilir ve sosyal güvenlik kurumlarından almakta oldukları aylıkları ... </t>
+  </si>
+  <si>
+    <t>sözleşmeli - kesilmez.</t>
+  </si>
+  <si>
+    <t>İlgili kanunlarına veya Cumhurbaşkanlığı kararnamelerine göre; öğrenim yapmak, yetiştirilmek, eğitilmek, bilgilerini artırmak, staj yapmak veya benzeri bir nedenle geçici süreli görevlendirilmek suretiyle, üç ay veya daha fazla süre ile yurtdışına gönderilen kamu personeli yurtdışında bulundukları sürenin ... katı kadar mecburi hizmetle yükümlüdürler. Bu şekilde yurt dışına gönderilecek personelden, örneği Maliye Bakanlığı tarafından hazırlanmış "Yüklenme Senedi ile Muteber İmzalı Müteselsil Kefalet Senedi" alınır.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Personelin mecburi hizmet yükümlülüğünü yerine getirmeden veya tamamlamadan görevinden ayrılması, müstafi sayılması ya da bir ceza ile görevine son verilmesi halinde, kendileri için kurumlarınca fiilen döviz olarak yapılmış olan her türlü masraflar aynı döviz cins ve miktarı üzerinden ..... Döviz borcu toplamından mecburi hizmetin tamamlanan kısmı için hesaplanan miktar indirilir. </t>
+  </si>
+  <si>
+    <t>borçlandırılır.</t>
+  </si>
+  <si>
+    <t>Uzman yardımcılığına atananlar, en az …. çalışmak ve istihdam edildikleri birimlerce belirlenecek konularda hazırlayacakları uzmanlık tezi, oluşturulacak tez jürisi tarafından kabul edilmek kaydıyla yeterlik sınavına girmeye hak kazanırlar.</t>
+  </si>
+  <si>
+    <t>üç yıl</t>
+  </si>
+  <si>
+    <t>Yarım zamanlı çalışma hakkının kullanımına ilişkin usul ve esaslar ile bu haktan yararlanamayacak memurları; hizmet sınıfı, kadro unvanı, kurum veya teşkilat bazında birlikte veya ayrı ayrı belirlemeye ….. yetkilidir.</t>
   </si>
 </sst>
 </file>
@@ -663,7 +1327,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="center"/>
@@ -686,6 +1350,10 @@
     </xf>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -814,7 +1482,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B62"/>
+  <dimension ref="A1:B194"/>
   <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="15.6"/>
   <cols>
     <col min="1" max="1" width="85.6640625" style="3" customWidth="1"/>
@@ -1318,6 +1986,1062 @@
         <v>116</v>
       </c>
     </row>
+    <row r="63" spans="1:2" ht="78">
+      <c r="A63" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="B63" s="3" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="64" spans="1:2" ht="31.2">
+      <c r="A64" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="B64" s="3" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="65" spans="1:2" ht="62.4">
+      <c r="A65" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="B65" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="66" spans="1:2">
+      <c r="A66" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="B66" s="3" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="67" spans="1:2" ht="62.4">
+      <c r="A67" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="B67" s="3" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="68" spans="1:2" ht="46.8">
+      <c r="A68" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="B68" s="3" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="69" spans="1:2" ht="46.8">
+      <c r="A69" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="B69" s="3" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="70" spans="1:2" ht="46.8">
+      <c r="A70" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="B70" s="3" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="71" spans="1:2" ht="46.8">
+      <c r="A71" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="B71" s="3" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="72" spans="1:2" ht="31.2">
+      <c r="A72" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="B72" s="3" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="73" spans="1:2">
+      <c r="A73" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="B73" s="3" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="74" spans="1:2" ht="31.2">
+      <c r="A74" s="4" t="s">
+        <v>136</v>
+      </c>
+      <c r="B74" s="3" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="75" spans="1:2">
+      <c r="A75" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="B75" s="3">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="76" spans="1:2" ht="31.2">
+      <c r="A76" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="B76" s="3" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="77" spans="1:2" ht="31.2">
+      <c r="A77" s="3" t="s">
+        <v>140</v>
+      </c>
+      <c r="B77" s="3" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="78" spans="1:2" ht="46.8">
+      <c r="A78" s="4" t="s">
+        <v>142</v>
+      </c>
+      <c r="B78" s="3" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="79" spans="1:2">
+      <c r="A79" s="9" t="s">
+        <v>144</v>
+      </c>
+      <c r="B79" s="3" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="80" spans="1:2" ht="46.8">
+      <c r="A80" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="B80" s="3" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="81" spans="1:2" ht="31.2">
+      <c r="A81" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="B81" s="3" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="82" spans="1:2" ht="31.2">
+      <c r="A82" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="B82" s="3" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="83" spans="1:2" ht="31.2">
+      <c r="A83" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="B83" s="3" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="84" spans="1:2">
+      <c r="A84" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="B84" s="3" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="85" spans="1:2" ht="46.8">
+      <c r="A85" s="6" t="s">
+        <v>156</v>
+      </c>
+      <c r="B85" s="3" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="86" spans="1:2" ht="62.4">
+      <c r="A86" s="4" t="s">
+        <v>158</v>
+      </c>
+      <c r="B86" s="3" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="87" spans="1:2" ht="31.2">
+      <c r="A87" s="4" t="s">
+        <v>159</v>
+      </c>
+      <c r="B87" s="3" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="88" spans="1:2" ht="78">
+      <c r="A88" s="1" t="s">
+        <v>161</v>
+      </c>
+      <c r="B88" s="3" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="89" spans="1:2" ht="46.8">
+      <c r="A89" s="6" t="s">
+        <v>163</v>
+      </c>
+      <c r="B89" s="3" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="90" spans="1:2" ht="46.8">
+      <c r="A90" s="10" t="s">
+        <v>165</v>
+      </c>
+      <c r="B90" s="3" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="91" spans="1:2" ht="46.8">
+      <c r="A91" s="7" t="s">
+        <v>166</v>
+      </c>
+      <c r="B91" s="3" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="92" spans="1:2" ht="46.8">
+      <c r="A92" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="B92" s="3" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="93" spans="1:2" ht="31.2">
+      <c r="A93" s="6" t="s">
+        <v>170</v>
+      </c>
+      <c r="B93" s="3" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="94" spans="1:2" ht="31.2">
+      <c r="A94" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="B94" s="3" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="95" spans="1:2" ht="31.2">
+      <c r="A95" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="B95" s="3" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="96" spans="1:2" ht="62.4">
+      <c r="A96" s="1" t="s">
+        <v>176</v>
+      </c>
+      <c r="B96" s="3" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="97" spans="1:2">
+      <c r="A97" s="1" t="s">
+        <v>177</v>
+      </c>
+      <c r="B97" s="3" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="98" spans="1:2">
+      <c r="A98" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="B98" s="3" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="99" spans="1:2">
+      <c r="A99" s="1" t="s">
+        <v>179</v>
+      </c>
+      <c r="B99" s="3" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="100" spans="1:2">
+      <c r="A100" s="2" t="s">
+        <v>180</v>
+      </c>
+      <c r="B100" s="3" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="101" spans="1:2">
+      <c r="A101" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="B101" s="3" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="102" spans="1:2">
+      <c r="A102" s="1" t="s">
+        <v>182</v>
+      </c>
+      <c r="B102" s="3" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="103" spans="1:2">
+      <c r="A103" s="1" t="s">
+        <v>183</v>
+      </c>
+      <c r="B103" s="3" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="104" spans="1:2">
+      <c r="A104" s="2" t="s">
+        <v>184</v>
+      </c>
+      <c r="B104" s="3" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="105" spans="1:2" ht="46.8">
+      <c r="A105" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="B105" s="3" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="106" spans="1:2" ht="31.2">
+      <c r="A106" s="3" t="s">
+        <v>187</v>
+      </c>
+      <c r="B106" s="3" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="107" spans="1:2">
+      <c r="A107" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="B107" s="3" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="108" spans="1:2" ht="31.2">
+      <c r="A108" s="3" t="s">
+        <v>189</v>
+      </c>
+      <c r="B108" s="3" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="109" spans="1:2">
+      <c r="A109" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="B109" s="3" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="110" spans="1:2">
+      <c r="A110" s="2" t="s">
+        <v>191</v>
+      </c>
+      <c r="B110" s="3" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="111" spans="1:2">
+      <c r="A111" s="1" t="s">
+        <v>192</v>
+      </c>
+      <c r="B111" s="3" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="112" spans="1:2">
+      <c r="A112" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="B112" s="3" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="113" spans="1:2" ht="31.2">
+      <c r="A113" s="3" t="s">
+        <v>194</v>
+      </c>
+      <c r="B113" s="3" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="114" spans="1:2">
+      <c r="A114" s="2" t="s">
+        <v>195</v>
+      </c>
+      <c r="B114" s="3" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="115" spans="1:2">
+      <c r="A115" s="1" t="s">
+        <v>196</v>
+      </c>
+      <c r="B115" s="3" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="116" spans="1:2">
+      <c r="A116" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="B116" s="3" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="117" spans="1:2" ht="31.2">
+      <c r="A117" s="3" t="s">
+        <v>198</v>
+      </c>
+      <c r="B117" s="3" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="118" spans="1:2">
+      <c r="A118" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="B118" s="3" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="119" spans="1:2" ht="46.8">
+      <c r="A119" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="B119" s="3" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="120" spans="1:2">
+      <c r="A120" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="B120" s="3" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="121" spans="1:2">
+      <c r="A121" s="2" t="s">
+        <v>203</v>
+      </c>
+      <c r="B121" s="3" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="122" spans="1:2">
+      <c r="A122" s="1" t="s">
+        <v>204</v>
+      </c>
+      <c r="B122" s="3" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="123" spans="1:2">
+      <c r="A123" s="2" t="s">
+        <v>205</v>
+      </c>
+      <c r="B123" s="3" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="124" spans="1:2" ht="31.2">
+      <c r="A124" s="3" t="s">
+        <v>206</v>
+      </c>
+      <c r="B124" s="3" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="125" spans="1:2" ht="31.2">
+      <c r="A125" s="3" t="s">
+        <v>207</v>
+      </c>
+      <c r="B125" s="3" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="126" spans="1:2" ht="31.2">
+      <c r="A126" s="3" t="s">
+        <v>208</v>
+      </c>
+      <c r="B126" s="3" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="127" spans="1:2" ht="46.8">
+      <c r="A127" s="2" t="s">
+        <v>210</v>
+      </c>
+      <c r="B127" s="3" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="128" spans="1:2" ht="46.8">
+      <c r="A128" s="2" t="s">
+        <v>212</v>
+      </c>
+      <c r="B128" s="3" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="129" spans="1:2" ht="46.8">
+      <c r="A129" s="1" t="s">
+        <v>213</v>
+      </c>
+      <c r="B129" s="3" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="130" spans="1:2" ht="46.8">
+      <c r="A130" s="2" t="s">
+        <v>214</v>
+      </c>
+      <c r="B130" s="3" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="131" spans="1:2" ht="46.8">
+      <c r="A131" s="3" t="s">
+        <v>215</v>
+      </c>
+      <c r="B131" s="3" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="132" spans="1:2" ht="46.8">
+      <c r="A132" s="2" t="s">
+        <v>216</v>
+      </c>
+      <c r="B132" s="3" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="133" spans="1:2" ht="46.8">
+      <c r="A133" s="3" t="s">
+        <v>217</v>
+      </c>
+      <c r="B133" s="3" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="134" spans="1:2" ht="46.8">
+      <c r="A134" s="3" t="s">
+        <v>218</v>
+      </c>
+      <c r="B134" s="3" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="135" spans="1:2" ht="46.8">
+      <c r="A135" s="2" t="s">
+        <v>219</v>
+      </c>
+      <c r="B135" s="3" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="136" spans="1:2" ht="46.8">
+      <c r="A136" s="2" t="s">
+        <v>220</v>
+      </c>
+      <c r="B136" s="3" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="137" spans="1:2" ht="46.8">
+      <c r="A137" s="3" t="s">
+        <v>221</v>
+      </c>
+      <c r="B137" s="3" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="138" spans="1:2" ht="62.4">
+      <c r="A138" s="3" t="s">
+        <v>222</v>
+      </c>
+      <c r="B138" s="3" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="139" spans="1:2" ht="46.8">
+      <c r="A139" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="B139" s="3" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="140" spans="1:2" ht="46.8">
+      <c r="A140" s="2" t="s">
+        <v>224</v>
+      </c>
+      <c r="B140" s="3" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="141" spans="1:2" ht="62.4">
+      <c r="A141" s="3" t="s">
+        <v>225</v>
+      </c>
+      <c r="B141" s="3" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="142" spans="1:2" ht="46.8">
+      <c r="A142" s="3" t="s">
+        <v>227</v>
+      </c>
+      <c r="B142" s="3" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="143" spans="1:2" ht="46.8">
+      <c r="A143" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="B143" s="3" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="144" spans="1:2" ht="46.8">
+      <c r="A144" s="2" t="s">
+        <v>229</v>
+      </c>
+      <c r="B144" s="3" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="145" spans="1:2" ht="46.8">
+      <c r="A145" s="3" t="s">
+        <v>230</v>
+      </c>
+      <c r="B145" s="3" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="146" spans="1:2" ht="46.8">
+      <c r="A146" s="9" t="s">
+        <v>231</v>
+      </c>
+      <c r="B146" s="3" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="147" spans="1:2" ht="46.8">
+      <c r="A147" s="3" t="s">
+        <v>232</v>
+      </c>
+      <c r="B147" s="3" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="148" spans="1:2" ht="46.8">
+      <c r="A148" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="B148" s="3" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="149" spans="1:2" ht="46.8">
+      <c r="A149" s="2" t="s">
+        <v>234</v>
+      </c>
+      <c r="B149" s="3" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="150" spans="1:2" ht="46.8">
+      <c r="A150" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="B150" s="3" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="151" spans="1:2" ht="46.8">
+      <c r="A151" s="2" t="s">
+        <v>236</v>
+      </c>
+      <c r="B151" s="3" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="152" spans="1:2" ht="46.8">
+      <c r="A152" s="3" t="s">
+        <v>237</v>
+      </c>
+      <c r="B152" s="3" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="153" spans="1:2" ht="46.8">
+      <c r="A153" s="1" t="s">
+        <v>238</v>
+      </c>
+      <c r="B153" s="3" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="154" spans="1:2" ht="46.8">
+      <c r="A154" s="3" t="s">
+        <v>240</v>
+      </c>
+      <c r="B154" s="3" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="155" spans="1:2" ht="31.2">
+      <c r="A155" s="1" t="s">
+        <v>242</v>
+      </c>
+      <c r="B155" s="3" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="156" spans="1:2" ht="31.2">
+      <c r="A156" s="3" t="s">
+        <v>244</v>
+      </c>
+      <c r="B156" s="3" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="157" spans="1:2" ht="31.2">
+      <c r="A157" s="3" t="s">
+        <v>246</v>
+      </c>
+      <c r="B157" s="3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="158" spans="1:2" ht="31.2">
+      <c r="A158" s="3" t="s">
+        <v>247</v>
+      </c>
+      <c r="B158" s="3" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="159" spans="1:2" ht="31.2">
+      <c r="A159" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="B159" s="3" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="160" spans="1:2" ht="31.2">
+      <c r="A160" s="3" t="s">
+        <v>250</v>
+      </c>
+      <c r="B160" s="3" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="161" spans="1:2" ht="31.2">
+      <c r="A161" s="1" t="s">
+        <v>252</v>
+      </c>
+      <c r="B161" s="3" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="162" spans="1:2" ht="46.8">
+      <c r="A162" s="1" t="s">
+        <v>253</v>
+      </c>
+      <c r="B162" s="3" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="163" spans="1:2" ht="46.8">
+      <c r="A163" s="1" t="s">
+        <v>255</v>
+      </c>
+      <c r="B163" s="3" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="164" spans="1:2" ht="46.8">
+      <c r="A164" s="1" t="s">
+        <v>257</v>
+      </c>
+      <c r="B164" s="3" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="165" spans="1:2" ht="31.2">
+      <c r="A165" s="1" t="s">
+        <v>259</v>
+      </c>
+      <c r="B165" s="3" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="166" spans="1:2" ht="46.8">
+      <c r="A166" s="3" t="s">
+        <v>261</v>
+      </c>
+      <c r="B166" s="3" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="167" spans="1:2" ht="62.4">
+      <c r="A167" s="4" t="s">
+        <v>263</v>
+      </c>
+      <c r="B167" s="3" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="168" spans="1:2" ht="46.8">
+      <c r="A168" s="3" t="s">
+        <v>265</v>
+      </c>
+      <c r="B168" s="3" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="169" spans="1:2" ht="46.8">
+      <c r="A169" s="6" t="s">
+        <v>266</v>
+      </c>
+      <c r="B169" s="3" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="170" spans="1:2" ht="31.2">
+      <c r="A170" s="6" t="s">
+        <v>268</v>
+      </c>
+      <c r="B170" s="3" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="171" spans="1:2" ht="31.2">
+      <c r="A171" s="6" t="s">
+        <v>270</v>
+      </c>
+      <c r="B171" s="3" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="172" spans="1:2" ht="124.8">
+      <c r="A172" s="2" t="s">
+        <v>272</v>
+      </c>
+      <c r="B172" s="3" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="173" spans="1:2" ht="31.2">
+      <c r="A173" s="1" t="s">
+        <v>274</v>
+      </c>
+      <c r="B173" s="3">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="174" spans="1:2" ht="31.2">
+      <c r="A174" s="3" t="s">
+        <v>275</v>
+      </c>
+      <c r="B174" s="3" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="175" spans="1:2" ht="31.2">
+      <c r="A175" s="3" t="s">
+        <v>277</v>
+      </c>
+      <c r="B175" s="3" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="176" spans="1:2" ht="31.2">
+      <c r="A176" s="3" t="s">
+        <v>279</v>
+      </c>
+      <c r="B176" s="2" t="s">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="177" spans="1:2">
+      <c r="A177" s="1" t="s">
+        <v>281</v>
+      </c>
+      <c r="B177" s="2" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="178" spans="1:2">
+      <c r="A178" s="1" t="s">
+        <v>283</v>
+      </c>
+      <c r="B178" s="2" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="179" spans="1:2" ht="46.8">
+      <c r="A179" s="3" t="s">
+        <v>285</v>
+      </c>
+      <c r="B179" s="3" t="s">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="180" spans="1:2" ht="46.8">
+      <c r="A180" s="3" t="s">
+        <v>287</v>
+      </c>
+      <c r="B180" s="3" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="181" spans="1:2" ht="46.8">
+      <c r="A181" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="B181" s="3" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="182" spans="1:2" ht="31.2">
+      <c r="A182" s="1" t="s">
+        <v>291</v>
+      </c>
+      <c r="B182" s="3" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="183" spans="1:2" ht="31.2">
+      <c r="A183" s="3" t="s">
+        <v>292</v>
+      </c>
+      <c r="B183" s="3" t="s">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="184" spans="1:2" ht="31.2">
+      <c r="A184" s="1" t="s">
+        <v>294</v>
+      </c>
+      <c r="B184" s="3" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="185" spans="1:2">
+      <c r="A185" s="2" t="s">
+        <v>297</v>
+      </c>
+      <c r="B185" s="3" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="186" spans="1:2">
+      <c r="A186" s="9" t="s">
+        <v>298</v>
+      </c>
+      <c r="B186" s="3" t="s">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="187" spans="1:2" ht="31.2">
+      <c r="A187" s="4" t="s">
+        <v>300</v>
+      </c>
+      <c r="B187" s="3" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="188" spans="1:2" ht="62.4">
+      <c r="A188" s="3" t="s">
+        <v>301</v>
+      </c>
+      <c r="B188" s="3" t="s">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="189" spans="1:2" ht="46.8">
+      <c r="A189" s="3" t="s">
+        <v>303</v>
+      </c>
+      <c r="B189" s="3" t="s">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="190" spans="1:2" ht="31.2">
+      <c r="A190" s="1" t="s">
+        <v>305</v>
+      </c>
+      <c r="B190" s="3" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="191" spans="1:2" ht="93.6">
+      <c r="A191" s="3" t="s">
+        <v>307</v>
+      </c>
+      <c r="B191" s="3" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="192" spans="1:2" ht="78">
+      <c r="A192" s="3" t="s">
+        <v>308</v>
+      </c>
+      <c r="B192" s="3" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="193" spans="1:2" ht="46.8">
+      <c r="A193" s="3" t="s">
+        <v>310</v>
+      </c>
+      <c r="B193" s="3" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="194" spans="1:2" ht="46.8">
+      <c r="A194" s="4" t="s">
+        <v>312</v>
+      </c>
+      <c r="B194" s="3" t="s">
+        <v>133</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.05277777777778" bottom="1.05277777777778" header="0.78749999999999998" footer="0.78749999999999998"/>
   <pageSetup paperSize="9" orientation="portrait" useFirstPageNumber="1" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>

</xml_diff>